<commit_message>
added a downloadable template. Fixed column number issues
</commit_message>
<xml_diff>
--- a/static/data/templates/chips_dataset_entry_template.xlsx
+++ b/static/data/templates/chips_dataset_entry_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TH282424\Rprojects\chips\static\data\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96A1C32F-8209-4D57-8ABA-B4287A8D0012}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B472D844-AA2C-4CBD-85C2-1DA2557BC5FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28704" yWindow="1116" windowWidth="21600" windowHeight="11124" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28704" yWindow="1116" windowWidth="21600" windowHeight="11124" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="5" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="165">
   <si>
     <t>137_1</t>
   </si>
@@ -527,13 +527,16 @@
   </si>
   <si>
     <t>9th to 11th c AD</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -918,7 +921,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7055C30-DE02-463C-97D2-34E9B4820BCC}">
   <dimension ref="A1:EH1"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.77734375" bestFit="1" customWidth="1"/>
@@ -1059,7 +1062,7 @@
     <col min="138" max="138" width="10.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:138">
+    <row r="1" spans="1:138" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -1483,7 +1486,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:EH10"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.88671875" bestFit="1" customWidth="1"/>
@@ -1594,7 +1597,7 @@
     <col min="138" max="138" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:138">
+    <row r="1" spans="1:138" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -2010,7 +2013,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="2" spans="1:138">
+    <row r="2" spans="1:138" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2305,8 +2308,17 @@
       <c r="EE2" t="s">
         <v>161</v>
       </c>
+      <c r="EF2" t="s">
+        <v>164</v>
+      </c>
+      <c r="EG2" t="s">
+        <v>164</v>
+      </c>
+      <c r="EH2" t="s">
+        <v>164</v>
+      </c>
     </row>
-    <row r="3" spans="1:138">
+    <row r="3" spans="1:138" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -2601,8 +2613,17 @@
       <c r="EE3" t="s">
         <v>161</v>
       </c>
+      <c r="EF3" t="s">
+        <v>164</v>
+      </c>
+      <c r="EG3" t="s">
+        <v>164</v>
+      </c>
+      <c r="EH3" t="s">
+        <v>164</v>
+      </c>
     </row>
-    <row r="4" spans="1:138">
+    <row r="4" spans="1:138" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -2897,8 +2918,17 @@
       <c r="EE4" t="s">
         <v>161</v>
       </c>
+      <c r="EF4" t="s">
+        <v>164</v>
+      </c>
+      <c r="EG4" t="s">
+        <v>164</v>
+      </c>
+      <c r="EH4" t="s">
+        <v>164</v>
+      </c>
     </row>
-    <row r="5" spans="1:138">
+    <row r="5" spans="1:138" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -3193,8 +3223,17 @@
       <c r="EE5" t="s">
         <v>161</v>
       </c>
+      <c r="EF5" t="s">
+        <v>164</v>
+      </c>
+      <c r="EG5" t="s">
+        <v>164</v>
+      </c>
+      <c r="EH5" t="s">
+        <v>164</v>
+      </c>
     </row>
-    <row r="6" spans="1:138">
+    <row r="6" spans="1:138" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -3489,8 +3528,17 @@
       <c r="EE6" t="s">
         <v>161</v>
       </c>
+      <c r="EF6" t="s">
+        <v>164</v>
+      </c>
+      <c r="EG6" t="s">
+        <v>164</v>
+      </c>
+      <c r="EH6" t="s">
+        <v>164</v>
+      </c>
     </row>
-    <row r="7" spans="1:138">
+    <row r="7" spans="1:138" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -3785,8 +3833,17 @@
       <c r="EE7" t="s">
         <v>161</v>
       </c>
+      <c r="EF7" t="s">
+        <v>164</v>
+      </c>
+      <c r="EG7" t="s">
+        <v>164</v>
+      </c>
+      <c r="EH7" t="s">
+        <v>164</v>
+      </c>
     </row>
-    <row r="8" spans="1:138">
+    <row r="8" spans="1:138" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -4081,8 +4138,17 @@
       <c r="EE8" t="s">
         <v>161</v>
       </c>
+      <c r="EF8" t="s">
+        <v>164</v>
+      </c>
+      <c r="EG8" t="s">
+        <v>164</v>
+      </c>
+      <c r="EH8" t="s">
+        <v>164</v>
+      </c>
     </row>
-    <row r="9" spans="1:138">
+    <row r="9" spans="1:138" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -4377,8 +4443,17 @@
       <c r="EE9" t="s">
         <v>161</v>
       </c>
+      <c r="EF9" t="s">
+        <v>164</v>
+      </c>
+      <c r="EG9" t="s">
+        <v>164</v>
+      </c>
+      <c r="EH9" t="s">
+        <v>164</v>
+      </c>
     </row>
-    <row r="10" spans="1:138">
+    <row r="10" spans="1:138" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -4672,6 +4747,15 @@
       </c>
       <c r="EE10" t="s">
         <v>161</v>
+      </c>
+      <c r="EF10" t="s">
+        <v>164</v>
+      </c>
+      <c r="EG10" t="s">
+        <v>164</v>
+      </c>
+      <c r="EH10" t="s">
+        <v>164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed a TSV related issue (empty columns)
</commit_message>
<xml_diff>
--- a/static/data/templates/chips_dataset_entry_template.xlsx
+++ b/static/data/templates/chips_dataset_entry_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TH282424\Rprojects\chips\static\data\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B472D844-AA2C-4CBD-85C2-1DA2557BC5FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BFE6921-8F5C-4E0F-AC04-856900D3506E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28704" yWindow="1116" windowWidth="21600" windowHeight="11124" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="166">
   <si>
     <t>137_1</t>
   </si>
@@ -530,6 +530,9 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>comment</t>
   </si>
 </sst>
 </file>
@@ -1485,7 +1488,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:EH10"/>
+  <dimension ref="A1:EI10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.77734375" bestFit="1" customWidth="1"/>
@@ -1597,7 +1600,7 @@
     <col min="138" max="138" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:138" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:139" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -2012,8 +2015,11 @@
       <c r="EH1" t="s">
         <v>145</v>
       </c>
+      <c r="EI1" t="s">
+        <v>165</v>
+      </c>
     </row>
-    <row r="2" spans="1:138" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:139" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2318,7 +2324,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="3" spans="1:138" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:139" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -2623,7 +2629,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="4" spans="1:138" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:139" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -2928,7 +2934,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="5" spans="1:138" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:139" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -3233,7 +3239,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="6" spans="1:138" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:139" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -3538,7 +3544,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="7" spans="1:138" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:139" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -3843,7 +3849,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="8" spans="1:138" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:139" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -4148,7 +4154,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="9" spans="1:138" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:139" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -4453,7 +4459,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="10" spans="1:138" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:139" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>

</xml_diff>